<commit_message>
Log 7 #projectdevelopment entries; add tasks 8-9 (RFI management system, Claire MoM follow-up)
</commit_message>
<xml_diff>
--- a/260729_K5M_Project Calendar.xlsx
+++ b/260729_K5M_Project Calendar.xlsx
@@ -27,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -93,6 +93,12 @@
       <color rgb="00E4572E"/>
       <sz val="7"/>
     </font>
+    <font>
+      <name val="Lato"/>
+      <color rgb="00292B2B"/>
+      <sz val="9"/>
+      <u val="single"/>
+    </font>
   </fonts>
   <fills count="12">
     <fill>
@@ -152,7 +158,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -232,11 +238,55 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thick">
+        <color rgb="00E4572E"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color rgb="00E4572E"/>
+      </right>
+      <top style="thick">
+        <color rgb="00E4572E"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color rgb="00E4572E"/>
+      </right>
+      <top style="thick">
+        <color rgb="00E4572E"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="00E4572E"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thick">
+        <color rgb="00E4572E"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="00E4572E"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -338,6 +388,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -745,6 +798,7 @@
           <t xml:space="preserve">  Deadline (red border)</t>
         </is>
       </c>
+      <c r="H2" s="41" t="n"/>
     </row>
     <row r="3" ht="26" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
@@ -2845,9 +2899,9 @@
           <t>⚑ SHD V00 parallel review &amp; feedback</t>
         </is>
       </c>
-      <c r="E28" s="17" t="n"/>
-      <c r="F28" s="17" t="n"/>
-      <c r="G28" s="18" t="n"/>
+      <c r="E28" s="42" t="n"/>
+      <c r="F28" s="42" t="n"/>
+      <c r="G28" s="41" t="n"/>
     </row>
     <row r="29" ht="34" customHeight="1">
       <c r="A29" s="14" t="n"/>
@@ -2941,8 +2995,8 @@
           <t>⚑ SHD V00 parallel review &amp; feedback</t>
         </is>
       </c>
-      <c r="B35" s="17" t="n"/>
-      <c r="C35" s="18" t="n"/>
+      <c r="B35" s="42" t="n"/>
+      <c r="C35" s="41" t="n"/>
       <c r="D35" s="21" t="inlineStr">
         <is>
           <t>SHD V01 drafting and issue</t>
@@ -3154,8 +3208,8 @@
           <t>⚑ SHD V00 parallel review &amp; feedback</t>
         </is>
       </c>
-      <c r="B7" s="17" t="n"/>
-      <c r="C7" s="18" t="n"/>
+      <c r="B7" s="42" t="n"/>
+      <c r="C7" s="41" t="n"/>
       <c r="D7" s="21" t="inlineStr">
         <is>
           <t>SHD V01 drafting and issue</t>
@@ -3424,9 +3478,9 @@
           <t>⚑ Signed GFP SHD Version 02</t>
         </is>
       </c>
-      <c r="E22" s="17" t="n"/>
-      <c r="F22" s="17" t="n"/>
-      <c r="G22" s="18" t="n"/>
+      <c r="E22" s="42" t="n"/>
+      <c r="F22" s="42" t="n"/>
+      <c r="G22" s="41" t="n"/>
     </row>
     <row r="23" ht="34" customHeight="1">
       <c r="A23" s="20" t="inlineStr">
@@ -3434,7 +3488,7 @@
           <t>⚑ Dispatch/delivery Round 1 sample box to Dubai</t>
         </is>
       </c>
-      <c r="B23" s="18" t="n"/>
+      <c r="B23" s="41" t="n"/>
       <c r="C23" s="21" t="inlineStr">
         <is>
           <t>Feedback round &amp; final approved material box</t>
@@ -3527,12 +3581,12 @@
           <t>⚑ Signed GFP SHD Version 02</t>
         </is>
       </c>
-      <c r="B28" s="17" t="n"/>
-      <c r="C28" s="17" t="n"/>
-      <c r="D28" s="17" t="n"/>
-      <c r="E28" s="17" t="n"/>
-      <c r="F28" s="17" t="n"/>
-      <c r="G28" s="18" t="n"/>
+      <c r="B28" s="42" t="n"/>
+      <c r="C28" s="42" t="n"/>
+      <c r="D28" s="42" t="n"/>
+      <c r="E28" s="42" t="n"/>
+      <c r="F28" s="42" t="n"/>
+      <c r="G28" s="41" t="n"/>
     </row>
     <row r="29" ht="34" customHeight="1">
       <c r="A29" s="16" t="inlineStr">
@@ -3638,12 +3692,12 @@
           <t>⚑ Signed GFP SHD Version 02</t>
         </is>
       </c>
-      <c r="B35" s="17" t="n"/>
-      <c r="C35" s="17" t="n"/>
-      <c r="D35" s="17" t="n"/>
-      <c r="E35" s="17" t="n"/>
-      <c r="F35" s="17" t="n"/>
-      <c r="G35" s="18" t="n"/>
+      <c r="B35" s="42" t="n"/>
+      <c r="C35" s="42" t="n"/>
+      <c r="D35" s="42" t="n"/>
+      <c r="E35" s="42" t="n"/>
+      <c r="F35" s="42" t="n"/>
+      <c r="G35" s="41" t="n"/>
     </row>
     <row r="36" ht="34" customHeight="1">
       <c r="A36" s="14" t="n"/>
@@ -3737,12 +3791,12 @@
           <t>⚑ Signed GFP SHD Version 02</t>
         </is>
       </c>
-      <c r="B42" s="17" t="n"/>
-      <c r="C42" s="17" t="n"/>
-      <c r="D42" s="17" t="n"/>
-      <c r="E42" s="17" t="n"/>
-      <c r="F42" s="17" t="n"/>
-      <c r="G42" s="18" t="n"/>
+      <c r="B42" s="42" t="n"/>
+      <c r="C42" s="42" t="n"/>
+      <c r="D42" s="42" t="n"/>
+      <c r="E42" s="42" t="n"/>
+      <c r="F42" s="42" t="n"/>
+      <c r="G42" s="41" t="n"/>
     </row>
     <row r="43" ht="34" customHeight="1">
       <c r="A43" s="24" t="inlineStr">
@@ -3771,8 +3825,8 @@
           <t>⚑ Signed FF&amp;E SHD V02 &amp; confirmed material package</t>
         </is>
       </c>
-      <c r="F44" s="17" t="n"/>
-      <c r="G44" s="18" t="n"/>
+      <c r="F44" s="42" t="n"/>
+      <c r="G44" s="41" t="n"/>
     </row>
     <row r="45" ht="34" customHeight="1">
       <c r="A45" s="14" t="n"/>
@@ -3991,12 +4045,12 @@
           <t>⚑ Signed GFP SHD Version 02</t>
         </is>
       </c>
-      <c r="B7" s="17" t="n"/>
-      <c r="C7" s="17" t="n"/>
-      <c r="D7" s="17" t="n"/>
-      <c r="E7" s="17" t="n"/>
-      <c r="F7" s="17" t="n"/>
-      <c r="G7" s="18" t="n"/>
+      <c r="B7" s="42" t="n"/>
+      <c r="C7" s="42" t="n"/>
+      <c r="D7" s="42" t="n"/>
+      <c r="E7" s="42" t="n"/>
+      <c r="F7" s="42" t="n"/>
+      <c r="G7" s="41" t="n"/>
     </row>
     <row r="8" ht="34" customHeight="1">
       <c r="A8" s="24" t="inlineStr">
@@ -4025,8 +4079,8 @@
           <t>⚑ Signed FF&amp;E SHD V02 &amp; confirmed material package</t>
         </is>
       </c>
-      <c r="F9" s="17" t="n"/>
-      <c r="G9" s="18" t="n"/>
+      <c r="F9" s="42" t="n"/>
+      <c r="G9" s="41" t="n"/>
     </row>
     <row r="10" ht="34" customHeight="1">
       <c r="A10" s="14" t="n"/>
@@ -4139,10 +4193,10 @@
           <t>⚑ Signed GFP SHD Version 02</t>
         </is>
       </c>
-      <c r="B15" s="17" t="n"/>
-      <c r="C15" s="17" t="n"/>
-      <c r="D15" s="17" t="n"/>
-      <c r="E15" s="18" t="n"/>
+      <c r="B15" s="42" t="n"/>
+      <c r="C15" s="42" t="n"/>
+      <c r="D15" s="42" t="n"/>
+      <c r="E15" s="41" t="n"/>
       <c r="F15" s="19" t="inlineStr">
         <is>
           <t>Send project update to internal WDCO K5M group</t>
@@ -4169,8 +4223,8 @@
           <t>⚑ Signed FF&amp;E SHD V02 &amp; confirmed material package</t>
         </is>
       </c>
-      <c r="B17" s="17" t="n"/>
-      <c r="C17" s="18" t="n"/>
+      <c r="B17" s="42" t="n"/>
+      <c r="C17" s="41" t="n"/>
       <c r="D17" s="16" t="inlineStr">
         <is>
           <t>FF&amp;E mock-up production, QC and packing</t>
@@ -4282,9 +4336,9 @@
           <t>⚑ Fit-out SHD V01 &amp; material-package approval</t>
         </is>
       </c>
-      <c r="E23" s="17" t="n"/>
-      <c r="F23" s="17" t="n"/>
-      <c r="G23" s="18" t="n"/>
+      <c r="E23" s="42" t="n"/>
+      <c r="F23" s="42" t="n"/>
+      <c r="G23" s="41" t="n"/>
     </row>
     <row r="24" ht="34" customHeight="1">
       <c r="A24" s="24" t="inlineStr">
@@ -4398,7 +4452,7 @@
           <t>⚑ Fit-out SHD V01 &amp; material-package approval</t>
         </is>
       </c>
-      <c r="B30" s="18" t="n"/>
+      <c r="B30" s="41" t="n"/>
       <c r="C30" s="16" t="inlineStr">
         <is>
           <t>Fit-out production, QC and packing</t>
@@ -6512,6 +6566,10 @@
           <t xml:space="preserve">  Deadline (red border)</t>
         </is>
       </c>
+      <c r="Q2" s="42" t="n"/>
+      <c r="R2" s="42" t="n"/>
+      <c r="S2" s="42" t="n"/>
+      <c r="T2" s="41" t="n"/>
     </row>
     <row r="3" ht="26" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
@@ -7814,53 +7872,177 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="40" t="n"/>
-      <c r="B6" s="40" t="n"/>
-      <c r="C6" s="40" t="n"/>
-      <c r="D6" s="40" t="n"/>
-      <c r="E6" s="40" t="n"/>
+      <c r="A6" s="40" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B6" s="40" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C6" s="40" t="inlineStr">
+        <is>
+          <t>COMM-C</t>
+        </is>
+      </c>
+      <c r="D6" s="40" t="inlineStr">
+        <is>
+          <t>Sent full Material Package email to G&amp;B, covering both FFE and Fitout.</t>
+        </is>
+      </c>
+      <c r="E6" s="43" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="40" t="n"/>
-      <c r="B7" s="40" t="n"/>
-      <c r="C7" s="40" t="n"/>
-      <c r="D7" s="40" t="n"/>
+      <c r="A7" s="40" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B7" s="40" t="inlineStr">
+        <is>
+          <t>WDCO Internal PM</t>
+        </is>
+      </c>
+      <c r="C7" s="40" t="inlineStr">
+        <is>
+          <t>WIPM</t>
+        </is>
+      </c>
+      <c r="D7" s="40" t="inlineStr">
+        <is>
+          <t>Project Calendar built (v1 + v2) — only aesthetic alignment left.</t>
+        </is>
+      </c>
       <c r="E7" s="40" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="40" t="n"/>
-      <c r="B8" s="40" t="n"/>
-      <c r="C8" s="40" t="n"/>
-      <c r="D8" s="40" t="n"/>
-      <c r="E8" s="40" t="n"/>
+      <c r="A8" s="40" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B8" s="40" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C8" s="40" t="inlineStr">
+        <is>
+          <t>RFI-C</t>
+        </is>
+      </c>
+      <c r="D8" s="40" t="inlineStr">
+        <is>
+          <t>Raised an RFI with the client regarding a high-resolution picture of GL-8.</t>
+        </is>
+      </c>
+      <c r="E8" s="43" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="40" t="n"/>
-      <c r="B9" s="40" t="n"/>
-      <c r="C9" s="40" t="n"/>
-      <c r="D9" s="40" t="n"/>
-      <c r="E9" s="40" t="n"/>
+      <c r="A9" s="40" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B9" s="40" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C9" s="40" t="inlineStr">
+        <is>
+          <t>FOSHD</t>
+        </is>
+      </c>
+      <c r="D9" s="40" t="inlineStr">
+        <is>
+          <t>Adil (architect) sent the DWG file of the entrance door.</t>
+        </is>
+      </c>
+      <c r="E9" s="43" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="40" t="n"/>
-      <c r="B10" s="40" t="n"/>
-      <c r="C10" s="40" t="n"/>
-      <c r="D10" s="40" t="n"/>
+      <c r="A10" s="40" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B10" s="40" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C10" s="40" t="inlineStr">
+        <is>
+          <t>WIPM</t>
+        </is>
+      </c>
+      <c r="D10" s="40" t="inlineStr">
+        <is>
+          <t>New lighting designer introduced; details to be updated in CONTACT_SHEET.md once confirmed.</t>
+        </is>
+      </c>
       <c r="E10" s="40" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="40" t="n"/>
-      <c r="B11" s="40" t="n"/>
-      <c r="C11" s="40" t="n"/>
-      <c r="D11" s="40" t="n"/>
+      <c r="A11" s="40" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B11" s="40" t="inlineStr">
+        <is>
+          <t>WDCO Internal PM</t>
+        </is>
+      </c>
+      <c r="C11" s="40" t="inlineStr"/>
+      <c r="D11" s="40" t="inlineStr">
+        <is>
+          <t>Meeting with Claire held — MoM to follow tomorrow.</t>
+        </is>
+      </c>
       <c r="E11" s="40" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="40" t="n"/>
-      <c r="B12" s="40" t="n"/>
-      <c r="C12" s="40" t="n"/>
-      <c r="D12" s="40" t="n"/>
-      <c r="E12" s="40" t="n"/>
+      <c r="A12" s="40" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B12" s="40" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C12" s="40" t="inlineStr">
+        <is>
+          <t>FOSHD</t>
+        </is>
+      </c>
+      <c r="D12" s="40" t="inlineStr">
+        <is>
+          <t>Closed fit-out RFIs with assigned actions; informed the client, will branch out further via email.</t>
+        </is>
+      </c>
+      <c r="E12" s="43" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="40" t="n"/>
@@ -8110,6 +8292,12 @@
       <formula1>"Project Scope,Project Schedule,Compliance Collection,FFE SHD,Material Package FFE,Material Package Fitout,Specifications from client,RFI - Client, Internal, Production Partner,Fitout SHD,COC Management,Communication Management - Internal, Production Partner, Client,Site Survey Planning"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId4"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Log lighting-designer email + new RFI (due 6 Aug) into Development Log, Data tab, August month grid, and Hard Milestones
</commit_message>
<xml_diff>
--- a/260729_K5M_Project Calendar.xlsx
+++ b/260729_K5M_Project Calendar.xlsx
@@ -756,7 +756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2449,6 +2449,37 @@
           <t>2026-12-31</t>
         </is>
       </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B54" s="8" t="inlineStr"/>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>RFI with lighting designer must be closed</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>Raised 30 Jul 2026.</t>
+        </is>
+      </c>
+      <c r="F54" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G54" s="8" t="inlineStr"/>
+      <c r="H54" s="8" t="inlineStr"/>
+      <c r="I54" s="8" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A5:I53"/>
@@ -3372,7 +3403,11 @@
       <c r="B16" s="18" t="n"/>
       <c r="C16" s="14" t="n"/>
       <c r="D16" s="14" t="n"/>
-      <c r="E16" s="14" t="n"/>
+      <c r="E16" s="15" t="inlineStr">
+        <is>
+          <t>⚑ RFI with lighting designer due</t>
+        </is>
+      </c>
       <c r="F16" s="19" t="inlineStr">
         <is>
           <t>Send project update to internal WDCO K5M group</t>
@@ -6782,7 +6817,7 @@
       <c r="L8" s="36" t="n">
         <v>5</v>
       </c>
-      <c r="M8" s="36" t="n">
+      <c r="M8" s="38" t="n">
         <v>6</v>
       </c>
       <c r="N8" s="36" t="n">
@@ -7405,7 +7440,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="14" customHeight="1">
+    <row r="21" ht="26" customHeight="1">
       <c r="A21" s="36" t="n">
         <v>20</v>
       </c>
@@ -7447,6 +7482,26 @@
       </c>
       <c r="O21" s="36" t="n">
         <v>24</v>
+      </c>
+      <c r="R21" s="33" t="inlineStr">
+        <is>
+          <t>06 Aug 2026</t>
+        </is>
+      </c>
+      <c r="S21" s="34" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="T21" s="33" t="inlineStr">
+        <is>
+          <t>RFI with lighting designer must be closed</t>
+        </is>
+      </c>
+      <c r="U21" s="33" t="inlineStr">
+        <is>
+          <t>Raised 30 Jul 2026.</t>
+        </is>
       </c>
     </row>
     <row r="22" ht="14" customHeight="1">
@@ -8045,17 +8100,49 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="40" t="n"/>
-      <c r="B13" s="40" t="n"/>
-      <c r="C13" s="40" t="n"/>
-      <c r="D13" s="40" t="n"/>
+      <c r="A13" s="40" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B13" s="40" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C13" s="40" t="inlineStr">
+        <is>
+          <t>Communication Management - Client</t>
+        </is>
+      </c>
+      <c r="D13" s="40" t="inlineStr">
+        <is>
+          <t>Sent introduction email to the new lighting designer.</t>
+        </is>
+      </c>
       <c r="E13" s="40" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="40" t="n"/>
-      <c r="B14" s="40" t="n"/>
-      <c r="C14" s="40" t="n"/>
-      <c r="D14" s="40" t="n"/>
+      <c r="A14" s="40" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B14" s="40" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C14" s="40" t="inlineStr">
+        <is>
+          <t>RFI - Client</t>
+        </is>
+      </c>
+      <c r="D14" s="40" t="inlineStr">
+        <is>
+          <t>Raised a new RFI with the lighting designer — must close by 6 Aug 2026.</t>
+        </is>
+      </c>
       <c r="E14" s="40" t="n"/>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
Log status-update email to Gisela; add follow-up + RFI tracking system tasks; update RFI task to In Progress
</commit_message>
<xml_diff>
--- a/260729_K5M_Project Calendar.xlsx
+++ b/260729_K5M_Project Calendar.xlsx
@@ -8146,11 +8146,31 @@
       <c r="E14" s="40" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="40" t="n"/>
-      <c r="B15" s="40" t="n"/>
-      <c r="C15" s="40" t="n"/>
-      <c r="D15" s="40" t="n"/>
-      <c r="E15" s="40" t="n"/>
+      <c r="A15" s="40" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B15" s="40" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C15" s="40" t="inlineStr">
+        <is>
+          <t>RFI - Client</t>
+        </is>
+      </c>
+      <c r="D15" s="40" t="inlineStr">
+        <is>
+          <t>Sent lighting designer (Gisela Steiger) a full status update on both scopes, referencing the still-open FF&amp;E lighting RFI directly.</t>
+        </is>
+      </c>
+      <c r="E15" s="43" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="40" t="n"/>
@@ -8384,6 +8404,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add BOQ scope gap meeting agenda (3 Aug); log to Task Tracker, Calendar, and Hard Milestones
</commit_message>
<xml_diff>
--- a/260729_K5M_Project Calendar.xlsx
+++ b/260729_K5M_Project Calendar.xlsx
@@ -756,7 +756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I54"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2480,6 +2480,37 @@
       <c r="G54" s="8" t="inlineStr"/>
       <c r="H54" s="8" t="inlineStr"/>
       <c r="I54" s="8" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B55" s="8" t="inlineStr"/>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>BOQ scope gap meeting — all stakeholders</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>Agenda: stone arch/wardrobe/fitted sofa, suspended glass light over basin, hardware &amp; bathroom fittings.</t>
+        </is>
+      </c>
+      <c r="F55" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G55" s="8" t="inlineStr"/>
+      <c r="H55" s="8" t="inlineStr"/>
+      <c r="I55" s="8" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A5:I53"/>
@@ -3430,7 +3461,11 @@
     </row>
     <row r="18" ht="34" customHeight="1">
       <c r="A18" s="14" t="n"/>
-      <c r="B18" s="14" t="n"/>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>⚑ BOQ scope gap meeting</t>
+        </is>
+      </c>
       <c r="C18" s="14" t="n"/>
       <c r="D18" s="14" t="n"/>
       <c r="E18" s="14" t="n"/>
@@ -6808,7 +6843,7 @@
       <c r="I8" s="36" t="n">
         <v>2</v>
       </c>
-      <c r="J8" s="36" t="n">
+      <c r="J8" s="38" t="n">
         <v>3</v>
       </c>
       <c r="K8" s="36" t="n">
@@ -7504,7 +7539,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="14" customHeight="1">
+    <row r="22" ht="26" customHeight="1">
       <c r="A22" s="36" t="n">
         <v>27</v>
       </c>
@@ -7540,6 +7575,26 @@
       </c>
       <c r="O22" s="36" t="n">
         <v>31</v>
+      </c>
+      <c r="R22" s="33" t="inlineStr">
+        <is>
+          <t>03 Aug 2026</t>
+        </is>
+      </c>
+      <c r="S22" s="34" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="T22" s="33" t="inlineStr">
+        <is>
+          <t>BOQ scope gap meeting — all stakeholders</t>
+        </is>
+      </c>
+      <c r="U22" s="33" t="inlineStr">
+        <is>
+          <t>Agenda: see meetings/260803_K5M_Meeting_BOQ_Scope_Gap.</t>
+        </is>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1">
@@ -8173,10 +8228,26 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="40" t="n"/>
-      <c r="B16" s="40" t="n"/>
-      <c r="C16" s="40" t="n"/>
-      <c r="D16" s="40" t="n"/>
+      <c r="A16" s="40" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B16" s="40" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C16" s="40" t="inlineStr">
+        <is>
+          <t>Project Scope</t>
+        </is>
+      </c>
+      <c r="D16" s="40" t="inlineStr">
+        <is>
+          <t>BOQ scope gap meeting confirmed for Monday 3 Aug — agenda: stone arch over wardrobe/fitted sofa, suspended glass light over basin, hardware &amp; bathroom fittings.</t>
+        </is>
+      </c>
       <c r="E16" s="40" t="n"/>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
Log 30 Jul project developments (H&T material package follow-up, Valentine/G&B sample-photo request, SketchUp model started, BOQ agenda draft, Ariel pause); update Task Tracker accordingly; correct remaining un-fixed Umbrella Task abbreviations in Development Log (WIPM, FOSHD -> full names)
</commit_message>
<xml_diff>
--- a/260729_K5M_Project Calendar.xlsx
+++ b/260729_K5M_Project Calendar.xlsx
@@ -7994,7 +7994,7 @@
       </c>
       <c r="C6" s="40" t="inlineStr">
         <is>
-          <t>COMM-C</t>
+          <t>Communication Management - Client</t>
         </is>
       </c>
       <c r="D6" s="40" t="inlineStr">
@@ -8021,7 +8021,7 @@
       </c>
       <c r="C7" s="40" t="inlineStr">
         <is>
-          <t>WIPM</t>
+          <t>WDCO Internal Project Management</t>
         </is>
       </c>
       <c r="D7" s="40" t="inlineStr">
@@ -8044,7 +8044,7 @@
       </c>
       <c r="C8" s="40" t="inlineStr">
         <is>
-          <t>RFI-C</t>
+          <t>RFI - Client</t>
         </is>
       </c>
       <c r="D8" s="40" t="inlineStr">
@@ -8071,7 +8071,7 @@
       </c>
       <c r="C9" s="40" t="inlineStr">
         <is>
-          <t>FOSHD</t>
+          <t>Fitout SHD</t>
         </is>
       </c>
       <c r="D9" s="40" t="inlineStr">
@@ -8098,7 +8098,7 @@
       </c>
       <c r="C10" s="40" t="inlineStr">
         <is>
-          <t>WIPM</t>
+          <t>WDCO Internal Project Management</t>
         </is>
       </c>
       <c r="D10" s="40" t="inlineStr">
@@ -8140,7 +8140,7 @@
       </c>
       <c r="C12" s="40" t="inlineStr">
         <is>
-          <t>FOSHD</t>
+          <t>Fitout SHD</t>
         </is>
       </c>
       <c r="D12" s="40" t="inlineStr">
@@ -8251,38 +8251,118 @@
       <c r="E16" s="40" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="40" t="n"/>
-      <c r="B17" s="40" t="n"/>
-      <c r="C17" s="40" t="n"/>
-      <c r="D17" s="40" t="n"/>
+      <c r="A17" s="40" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B17" s="40" t="inlineStr">
+        <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="C17" s="40" t="inlineStr">
+        <is>
+          <t>Material Package FFE</t>
+        </is>
+      </c>
+      <c r="D17" s="40" t="inlineStr">
+        <is>
+          <t>H&amp;T followed up on the Material Package — confirmed today's review meeting at 10am to go through it together.</t>
+        </is>
+      </c>
       <c r="E17" s="40" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="40" t="n"/>
-      <c r="B18" s="40" t="n"/>
-      <c r="C18" s="40" t="n"/>
-      <c r="D18" s="40" t="n"/>
+      <c r="A18" s="40" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B18" s="40" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C18" s="40" t="inlineStr">
+        <is>
+          <t>Material Package Fitout</t>
+        </is>
+      </c>
+      <c r="D18" s="40" t="inlineStr">
+        <is>
+          <t>Valentine (design team) emailed confirming she's clear on the material package and asked for sample photos if possible. Will try to resolve this in today's H&amp;T meeting; if not, will reply to her directly by 1pm today.</t>
+        </is>
+      </c>
       <c r="E18" s="40" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="40" t="n"/>
-      <c r="B19" s="40" t="n"/>
-      <c r="C19" s="40" t="n"/>
-      <c r="D19" s="40" t="n"/>
+      <c r="A19" s="40" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B19" s="40" t="inlineStr">
+        <is>
+          <t>WDCO Internal PM</t>
+        </is>
+      </c>
+      <c r="C19" s="40" t="inlineStr">
+        <is>
+          <t>WDCO Internal Project Management</t>
+        </is>
+      </c>
+      <c r="D19" s="40" t="inlineStr">
+        <is>
+          <t>Started work on the Google SketchUp model for the project briefing.</t>
+        </is>
+      </c>
       <c r="E19" s="40" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="40" t="n"/>
-      <c r="B20" s="40" t="n"/>
-      <c r="C20" s="40" t="n"/>
-      <c r="D20" s="40" t="n"/>
+      <c r="A20" s="40" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B20" s="40" t="inlineStr">
+        <is>
+          <t>WDCO Internal PM</t>
+        </is>
+      </c>
+      <c r="C20" s="40" t="inlineStr">
+        <is>
+          <t>Project Scope</t>
+        </is>
+      </c>
+      <c r="D20" s="40" t="inlineStr">
+        <is>
+          <t>Drafted a basic agenda for the BOQ scope gap meeting (Monday, 3 Aug) — alongside the formal agenda doc already prepared and stored in the project management folder.</t>
+        </is>
+      </c>
       <c r="E20" s="40" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="40" t="n"/>
-      <c r="B21" s="40" t="n"/>
-      <c r="C21" s="40" t="n"/>
-      <c r="D21" s="40" t="n"/>
+      <c r="A21" s="40" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B21" s="40" t="inlineStr">
+        <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="C21" s="40" t="inlineStr">
+        <is>
+          <t>Fitout SHD</t>
+        </is>
+      </c>
+      <c r="D21" s="40" t="inlineStr">
+        <is>
+          <t>Sent Ariel all details for the fit-out drawings; Claire has asked to pause this, as a new team joinee starts Monday (3 Aug) — will assess whether he can take this on before deciding who owns the work.</t>
+        </is>
+      </c>
       <c r="E21" s="40" t="n"/>
     </row>
     <row r="22">

</xml_diff>

<commit_message>
projectdevelopment: log stone reference image request to Valentine (design team)
</commit_message>
<xml_diff>
--- a/260729_K5M_Project Calendar.xlsx
+++ b/260729_K5M_Project Calendar.xlsx
@@ -27,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -98,6 +98,13 @@
       <color rgb="00292B2B"/>
       <sz val="9"/>
       <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="12">
@@ -283,10 +290,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -391,9 +399,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -8366,11 +8376,31 @@
       <c r="E21" s="40" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="40" t="n"/>
-      <c r="B22" s="40" t="n"/>
-      <c r="C22" s="40" t="n"/>
-      <c r="D22" s="40" t="n"/>
-      <c r="E22" s="40" t="n"/>
+      <c r="A22" s="40" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B22" s="40" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C22" s="40" t="inlineStr">
+        <is>
+          <t>Material Package FFE</t>
+        </is>
+      </c>
+      <c r="D22" s="40" t="inlineStr">
+        <is>
+          <t>Sent Valentine (design team) a request for stone reference images for three FFE stones (Calacatta Oro, Taj Mahal, Alabaster) — attached internet-sourced reference images based on the names she provided, purely to align on general visual direction before sample development.</t>
+        </is>
+      </c>
+      <c r="E22" s="44" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="40" t="n"/>
@@ -8556,6 +8586,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Log 3-6 Aug Project Development entries (BOQ gap meeting, Khamille meeting, Abdellatif, SHD01 review, Resti)
</commit_message>
<xml_diff>
--- a/260729_K5M_Project Calendar.xlsx
+++ b/260729_K5M_Project Calendar.xlsx
@@ -8403,94 +8403,302 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="40" t="n"/>
-      <c r="B23" s="40" t="n"/>
-      <c r="C23" s="40" t="n"/>
-      <c r="D23" s="40" t="n"/>
+      <c r="A23" s="40" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B23" s="40" t="inlineStr">
+        <is>
+          <t>WDCO Internal PM</t>
+        </is>
+      </c>
+      <c r="C23" s="40" t="inlineStr">
+        <is>
+          <t>Project Scope</t>
+        </is>
+      </c>
+      <c r="D23" s="40" t="inlineStr">
+        <is>
+          <t>BOQ gap meeting held. Decided: Resti's stone arch calculation to be documented clearly and incorporated into the existing scope-gap findings.</t>
+        </is>
+      </c>
       <c r="E23" s="40" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="40" t="n"/>
-      <c r="B24" s="40" t="n"/>
-      <c r="C24" s="40" t="n"/>
-      <c r="D24" s="40" t="n"/>
+      <c r="A24" s="40" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B24" s="40" t="inlineStr">
+        <is>
+          <t>WDCO Internal PM</t>
+        </is>
+      </c>
+      <c r="C24" s="40" t="inlineStr">
+        <is>
+          <t>Communication Management - Internal</t>
+        </is>
+      </c>
+      <c r="D24" s="40" t="inlineStr">
+        <is>
+          <t>Decided to send a consolidated BOQ-changes email (the gap, the difference) to Filippo Sona (WDCO co-founder/main partner) to handle from there.</t>
+        </is>
+      </c>
       <c r="E24" s="40" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="40" t="n"/>
-      <c r="B25" s="40" t="n"/>
-      <c r="C25" s="40" t="n"/>
-      <c r="D25" s="40" t="n"/>
+      <c r="A25" s="40" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B25" s="40" t="inlineStr">
+        <is>
+          <t>WDCO Internal PM</t>
+        </is>
+      </c>
+      <c r="C25" s="40" t="inlineStr">
+        <is>
+          <t>Logistics</t>
+        </is>
+      </c>
+      <c r="D25" s="40" t="inlineStr">
+        <is>
+          <t>Decided to email Maria (WDCO logistics) for container requirements so booking can proceed right away.</t>
+        </is>
+      </c>
       <c r="E25" s="40" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="40" t="n"/>
-      <c r="B26" s="40" t="n"/>
-      <c r="C26" s="40" t="n"/>
-      <c r="D26" s="40" t="n"/>
+      <c r="A26" s="40" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B26" s="40" t="inlineStr">
+        <is>
+          <t>WDCO Internal PM</t>
+        </is>
+      </c>
+      <c r="C26" s="40" t="inlineStr">
+        <is>
+          <t>Project Scope</t>
+        </is>
+      </c>
+      <c r="D26" s="40" t="inlineStr">
+        <is>
+          <t>Decided to build a new Fitout Scope document — fully defined, with a "Doubts" section for removable/uncertain items. Resolves the long-pending Fitout base-scope file (Hard Rule 14).</t>
+        </is>
+      </c>
       <c r="E26" s="40" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="40" t="n"/>
-      <c r="B27" s="40" t="n"/>
-      <c r="C27" s="40" t="n"/>
-      <c r="D27" s="40" t="n"/>
+      <c r="A27" s="40" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B27" s="40" t="inlineStr">
+        <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="C27" s="40" t="inlineStr">
+        <is>
+          <t>Fitout SHD</t>
+        </is>
+      </c>
+      <c r="D27" s="40" t="inlineStr">
+        <is>
+          <t>Decided to schedule a fitout scope meeting with H&amp;T ASAP.</t>
+        </is>
+      </c>
       <c r="E27" s="40" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="40" t="n"/>
-      <c r="B28" s="40" t="n"/>
-      <c r="C28" s="40" t="n"/>
-      <c r="D28" s="40" t="n"/>
+      <c r="A28" s="40" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B28" s="40" t="inlineStr">
+        <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="C28" s="40" t="inlineStr">
+        <is>
+          <t>Fitout SHD</t>
+        </is>
+      </c>
+      <c r="D28" s="40" t="inlineStr">
+        <is>
+          <t>Ariel to confirm which fitout drawings are shareable — deadline 7 Aug.</t>
+        </is>
+      </c>
       <c r="E28" s="40" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="40" t="n"/>
-      <c r="B29" s="40" t="n"/>
-      <c r="C29" s="40" t="n"/>
-      <c r="D29" s="40" t="n"/>
+      <c r="A29" s="40" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B29" s="40" t="inlineStr">
+        <is>
+          <t>WDCO Internal PM</t>
+        </is>
+      </c>
+      <c r="C29" s="40" t="inlineStr">
+        <is>
+          <t>Site Survey Planning</t>
+        </is>
+      </c>
+      <c r="D29" s="40" t="inlineStr">
+        <is>
+          <t>Site visit timing remains under ambiguity; white-box photos and a post-site-survey deliverable required regardless.</t>
+        </is>
+      </c>
       <c r="E29" s="40" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="40" t="n"/>
-      <c r="B30" s="40" t="n"/>
-      <c r="C30" s="40" t="n"/>
-      <c r="D30" s="40" t="n"/>
+      <c r="A30" s="40" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B30" s="40" t="inlineStr">
+        <is>
+          <t>WDCO Internal PM</t>
+        </is>
+      </c>
+      <c r="C30" s="40" t="inlineStr">
+        <is>
+          <t>Compliance Collection</t>
+        </is>
+      </c>
+      <c r="D30" s="40" t="inlineStr">
+        <is>
+          <t>Decided to compile all compliance documents received into a single consolidated record.</t>
+        </is>
+      </c>
       <c r="E30" s="40" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="40" t="n"/>
-      <c r="B31" s="40" t="n"/>
-      <c r="C31" s="40" t="n"/>
-      <c r="D31" s="40" t="n"/>
+      <c r="A31" s="40" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B31" s="40" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C31" s="40" t="inlineStr">
+        <is>
+          <t>Compliance Collection</t>
+        </is>
+      </c>
+      <c r="D31" s="40" t="inlineStr">
+        <is>
+          <t>Compliance documents request sent to Abdellatif Menbar (per Claire's direction); targeting close by 10 Aug.</t>
+        </is>
+      </c>
       <c r="E31" s="40" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="40" t="n"/>
-      <c r="B32" s="40" t="n"/>
-      <c r="C32" s="40" t="n"/>
-      <c r="D32" s="40" t="n"/>
+      <c r="A32" s="40" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B32" s="40" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C32" s="40" t="inlineStr">
+        <is>
+          <t>Fitout SHD</t>
+        </is>
+      </c>
+      <c r="D32" s="40" t="inlineStr">
+        <is>
+          <t>Sent Abdellatif Menbar the substructure requirements per Claire's direction; further discussion ongoing via email with the client team.</t>
+        </is>
+      </c>
       <c r="E32" s="40" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="40" t="n"/>
-      <c r="B33" s="40" t="n"/>
-      <c r="C33" s="40" t="n"/>
-      <c r="D33" s="40" t="n"/>
+      <c r="A33" s="40" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B33" s="40" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="C33" s="40" t="inlineStr">
+        <is>
+          <t>Material Package FFE</t>
+        </is>
+      </c>
+      <c r="D33" s="40" t="inlineStr">
+        <is>
+          <t>Met with Khamille on sample development — agreed swatch quantities per material (Fitout: 5 Stone/3 Wood/4 Metal/4 Glass/3 Fabric/1 Seating; FFE: 2 Wood/5 Metal/2 Glass/3 Stone/10 Fabric) and swatch sizes (Fabric/Wood/Glass 14x10cm, Metal 10x7cm), plus a wood-swatch construction spec (real wood + associated veneer). Already shared with H&amp;T. Presentation concept for the swatch box still to be developed.</t>
+        </is>
+      </c>
       <c r="E33" s="40" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="40" t="n"/>
-      <c r="B34" s="40" t="n"/>
-      <c r="C34" s="40" t="n"/>
-      <c r="D34" s="40" t="n"/>
+      <c r="A34" s="40" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B34" s="40" t="inlineStr">
+        <is>
+          <t>WDCO Internal PM</t>
+        </is>
+      </c>
+      <c r="C34" s="40" t="inlineStr">
+        <is>
+          <t>FFE SHD</t>
+        </is>
+      </c>
+      <c r="D34" s="40" t="inlineStr">
+        <is>
+          <t>Internal FFE Shop Drawing (SHD01) review meeting held, 10:30am. MOM to follow.</t>
+        </is>
+      </c>
       <c r="E34" s="40" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="40" t="n"/>
-      <c r="B35" s="40" t="n"/>
-      <c r="C35" s="40" t="n"/>
-      <c r="D35" s="40" t="n"/>
+      <c r="A35" s="40" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B35" s="40" t="inlineStr">
+        <is>
+          <t>WDCO Internal PM</t>
+        </is>
+      </c>
+      <c r="C35" s="40" t="inlineStr">
+        <is>
+          <t>Project Scope</t>
+        </is>
+      </c>
+      <c r="D35" s="40" t="inlineStr">
+        <is>
+          <t>Resti completed the stone arch BOQ gap calculation requested — write-up still to follow.</t>
+        </is>
+      </c>
       <c r="E35" s="40" t="n"/>
     </row>
     <row r="36">

</xml_diff>